<commit_message>
Verify PA AORO contacts and stop using purchasing inboxes.
RTKL recipients are the county Open Records officers from live Right-to-Know pages. Washington has no published AORO email and is marked UNVERIFIED.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/output/pa_followup/PA_procurement_contacts.xlsx
+++ b/data/output/pa_followup/PA_procurement_contacts.xlsx
@@ -427,20 +427,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,50 +456,75 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>jurisdiction</t>
+          <t>aoro_status</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>aoro_officer</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>officer</t>
+          <t>aoro_title</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>aoro_email</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>aoro_phone</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>aoro_address</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>source_url</t>
+          <t>aoro_source_url</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>verified_on</t>
+          <t>aoro_name_source_url</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>purchasing_officer</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>purchasing_title</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>purchasing_email</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>purchasing_phone</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>purchasing_source_url</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>fy2027_contracted_tons</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -508,52 +538,77 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Allegheny County</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Jessica Garofolo</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Open Records Officer</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>openrecords@alleghenycounty.us</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>412-350-6109</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>County Office Building, 542 Forbes Avenue, Room 101 Mezzanine, Pittsburgh, PA 15219</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.alleghenycounty.us/Government/Records/Open-Records</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.openrecords.pa.gov/RTKL/AOROInfo.cfm?id=39</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Frank Alessio</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>Chief Purchasing Officer</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Frank Alessio</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>bidsupport@alleghenycounty.us</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>412-350-6918</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>County Office Building, 542 Forbes Avenue, Room 201, Pittsburgh, PA 15219</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>https://www.alleghenycounty.us/Projects-and-Initiatives/Doing-Business-with-Allegheny-County-Bids-and-Solicitations/Purchasing-and-Supplies</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>142820</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Department inbox published for purchasing correspondence (Bonfire is the bid portal).</t>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>County Open Records page (retrieved 10 Sep 2026) names Garofolo and publishes the email. PA OOR listing id=39 matches the name; OOR hides the mailbox behind CAPTCHA.</t>
         </is>
       </c>
     </row>
@@ -565,52 +620,77 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Westmoreland County</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Stephanie Paha</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Agency Open Records Officer</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>records@westmorelandcountypa.gov</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>724-830-3145</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Open Records Officer, 2 N. Main Street, Suite 103, Greensburg, PA 15601</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.westmorelandcountypa.gov/431/Open-Records-Request</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.openrecords.pa.gov/RTKL/AOROInfo.cfm?id=2804</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Charlie Varriano</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>Director of Purchasing</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Charlie Varriano</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>cvarrian@westmorelandcountypa.gov</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>724-830-3753</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2 N. Main Street, Suite 14, Greensburg, PA 15601</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>https://www.westmorelandcountypa.gov/Directory.aspx?DID=116</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>108199</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Published on the county purchasing staff directory.</t>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Email and office are on the county Right-to-Know page (retrieved 10 Sep 2026). The page does not print a personal name; Stephanie Paha is the registered AORO on PA OOR listing id=2804 (phone 724-830-3145). In-person filing is the Solicitor's Office at the same address. Do not use the 2008 Lucy Yakulis policy or older Greenwald listings.</t>
         </is>
       </c>
     </row>
@@ -622,52 +702,77 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Luzerne County</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Purchasing Department</t>
+          <t>Tess Reilly</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Open Records Officer — County Administration</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Admin-RTK@luzernecounty.org</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>570-820-6359</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Luzerne County Office of Law, 200 Old Train Station Rd., Wilkes-Barre, PA 18702</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.luzernecounty.org/427/Luzerne-County-Open-Records-Officers</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://www.openrecords.pa.gov/RTKL/AOROInfo.cfm?id=1801</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>Mary Ann Amesbury</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Director of Purchasing</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>Purchasing@LuzerneCounty.org</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>570-825-1501</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Penn Place Suite 203, 20 N Pennsylvania Avenue, Wilkes-Barre, PA 18711</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>https://www.luzernecounty.org/309/Purchasing</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>73599</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Use the department inbox. Director email is also posted (MaryAnn.Amesbury@luzernecounty.org).</t>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>County Open Records Officers page (retrieved 10 Sep 2026) lists Tess Reilly for Luzerne County Administration with Admin-RTK@luzernecounty.org. PA OOR listing id=1801 names Therese Reilly (same officer). Court and DA officers are separate and are not the recipient for purchasing/salt contracts.</t>
         </is>
       </c>
     </row>
@@ -679,52 +784,77 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Washington County</t>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Cynthia Griffin</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Chief Clerk and Agency Open Records Officer</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>724-228-6915</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>95 West Beau Street, Suite 605, Washington, PA 15301</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.washcopa.gov/chief-clerk</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.openrecords.pa.gov/RTKL/AOROInfo.cfm?id=2700</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Randy K. Vankirk</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>Director of Purchasing</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Randy K. Vankirk</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>purchasing@washingtoncopa.gov</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>724-228-6740</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Crossroads Center, 95 W. Beau St., Suite 430, Washington, PA 15301</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>https://www.washingtoncopa.gov/purchasing</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>66141</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Department inbox listed on the county purchasing page.</t>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Officer identity is on the Chief Clerk page (retrieved 10 Sep 2026) and PA OOR listing id=2700. No AORO email is published on that page; OOR hides it behind CAPTCHA. County RTK submissions are via the web form linked from the Chief Clerk page. Do not substitute purchasing@washingtoncopa.gov as the RTKL recipient.</t>
         </is>
       </c>
     </row>
@@ -736,48 +866,73 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Erie County</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Deanna Heasley</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>County Solicitor / Open Records Officer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DHeasley@eriecountypa.gov</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>814-451-6344</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Erie County Courthouse, 140 West Sixth Street, Suite 504, Erie, PA 16501</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://eriecountypa.gov/open-government/right-to-know-request/</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.openrecords.pa.gov/RTKL/AOROInfo.cfm?id=1216</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>Department of Procurement</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>procurement@eriecountypa.gov</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>814-451-6244</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Erie County Courthouse, 140 West Sixth Street, Room 106, Erie, PA 16501</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>https://eriecountypa.gov/departments/procurement/open-bids/</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>64036</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Department inbox listed on the county procurement page.</t>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>County Right-to-Know page (retrieved 10 Sep 2026) designates the County Solicitor as Open Records Officer and publishes DHeasley@eriecountypa.gov. PA OOR listing id=1216 names Deanna L. Heasley.</t>
         </is>
       </c>
     </row>
@@ -801,7 +956,7 @@
     <row r="1" ht="80" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Pilot: five Pennsylvania counties by FY2027 contracted tons on the statewide COSTARS award. Emails are department inboxes published on county websites (retrieved 10 Sep 2026). Default: python scripts/pa_followup.py writes this workbook and .eml drafts. Sending requires --send and SALTTRACKER_FOLLOWUP_CONFIRM=YES. IMAP forwarding of replies uses --poll-inbox.</t>
+          <t>Pilot: five Pennsylvania counties by FY2027 contracted tons. Primary recipient is the county Agency Open Records Officer (RTKL), verified 10 Sep 2026 from the county Right-to-Know page. Purchasing contacts are secondary only. Washington AORO email is UNVERIFIED (not published; use the county web form). Default: python scripts/pa_followup.py writes this workbook and .eml drafts. Sending requires --send and SALTTRACKER_FOLLOWUP_CONFIRM=YES and skips UNVERIFIED rows.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Route salt RTKs to central AOROs; skip Washington with a web form.
Procurement and Public Works have no published deputy ORO in any of the five counties. Washington stays unscrapeable by email; the row now has the DocuSign RTK form URL for manual filing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/output/pa_followup/PA_procurement_contacts.xlsx
+++ b/data/output/pa_followup/PA_procurement_contacts.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -444,8 +444,12 @@
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="25" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="27" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,10 +525,30 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>salt_holder_has_own_oro</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>salt_routing_cite</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>submission_method</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>rtk_web_form_url</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>fy2027_contracted_tons</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -603,12 +627,28 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>https://www.alleghenycounty.us/Government/Records/Open-Records</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>email, mail, fax, in-person, online</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
           <t>142820</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>County Open Records page (retrieved 10 Sep 2026) names Garofolo and publishes the email. PA OOR listing id=39 matches the name; OOR hides the mailbox behind CAPTCHA.</t>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Department list on the Open Records page (retrieved 10 Sep 2026) is BPAAR, Controller, Council, Courts, CYF, DA, Redevelopment, Sheriff, Treasurer. Purchasing and Public Works are not listed; 'All other requests' go to the Office of Open Records. County policy PDF requires written requests be addressed to the County Open Records Officer; department assistant OROs only forward internally. To: stays Garofolo. Policy: https://www.alleghenycounty.us/files/assets/county/v/1/government/records/documents/openrecordspolicy.pdf</t>
         </is>
       </c>
     </row>
@@ -685,12 +725,28 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>https://www.westmorelandcountypa.gov/431/Open-Records-Request</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>email, mail, fax, in-person</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
           <t>108199</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Email and office are on the county Right-to-Know page (retrieved 10 Sep 2026). The page does not print a personal name; Stephanie Paha is the registered AORO on PA OOR listing id=2804 (phone 724-830-3145). In-person filing is the Solicitor's Office at the same address. Do not use the 2008 Lucy Yakulis policy or older Greenwald listings.</t>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Open Records Request page (retrieved 10 Sep 2026) names a single Open Records Officer / Solicitor's Office intake. No Procurement or Public Works deputy ORO. Email the saved form to records@westmorelandcountypa.gov.</t>
         </is>
       </c>
     </row>
@@ -767,12 +823,28 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>https://www.luzernecounty.org/427/Luzerne-County-Open-Records-Officers</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>email, mail</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
           <t>73599</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>County Open Records Officers page (retrieved 10 Sep 2026) lists Tess Reilly for Luzerne County Administration with Admin-RTK@luzernecounty.org. PA OOR listing id=1801 names Therese Reilly (same officer). Court and DA officers are separate and are not the recipient for purchasing/salt contracts.</t>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Open Records Officers page (retrieved 10 Sep 2026) splits Court, DA, Retirement Board, and County Administration. No Procurement or Public Works officer. Salt/purchasing records are Administration → Tess Reilly / Admin-RTK@luzernecounty.org.</t>
         </is>
       </c>
     </row>
@@ -849,12 +921,32 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>https://www.washcopa.gov/chief-clerk</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>web form, mail</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>https://apps.docusign.com/webforms/us/e9ef3ac01d292d1668e822e4f2370457</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
           <t>66141</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Officer identity is on the Chief Clerk page (retrieved 10 Sep 2026) and PA OOR listing id=2700. No AORO email is published on that page; OOR hides it behind CAPTCHA. County RTK submissions are via the web form linked from the Chief Clerk page. Do not substitute purchasing@washingtoncopa.gov as the RTKL recipient.</t>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>SKIP automated email. No AORO email on the Chief Clerk page (retrieved 10 Sep 2026). File manually via the 'Right to Know Request Web Form' linked from that page (DocuSign, HTTP 200 on 10 Sep 2026) or mail the Chief Clerk. No Procurement/Public Works deputy ORO on that page. Do not guess an email.</t>
         </is>
       </c>
     </row>
@@ -927,12 +1019,28 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>https://eriecountypa.gov/open-government/right-to-know-request/</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>email, mail, fax, in-person</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
           <t>64036</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>County Right-to-Know page (retrieved 10 Sep 2026) designates the County Solicitor as Open Records Officer and publishes DHeasley@eriecountypa.gov. PA OOR listing id=1216 names Deanna L. Heasley.</t>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Right-to-Know page (retrieved 10 Sep 2026) lists deputy OROs for Clerk of Records, Controller, Coroner, Council, Courts, DA, OCY, Sheriff. Procurement and Public Works are not on that deputy list. Requests with no deputy go to the County Solicitor (Administration). To: stays DHeasley@eriecountypa.gov.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record Washington’s Right-to-Know route as mail-only.
The DocuSign URL is UNCONFIRMED; do not email an unpublished AORO address.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/output/pa_followup/PA_procurement_contacts.xlsx
+++ b/data/output/pa_followup/PA_procurement_contacts.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>web form, mail</t>
+          <t>mail</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>SKIP automated email. No AORO email on the Chief Clerk page (retrieved 10 Sep 2026). File manually via the 'Right to Know Request Web Form' linked from that page (DocuSign, HTTP 200 on 10 Sep 2026) or mail the Chief Clerk. No Procurement/Public Works deputy ORO on that page. Do not guess an email.</t>
+          <t>SKIP automated email. No AORO email on the Chief Clerk page (retrieved 10 Sep 2026). Primary route: mail Cynthia Griffin, 95 West Beau Street, Suite 605, Washington, PA 15301. The Chief Clerk page links a DocuSign URL, but a 200 only loads the generic Docusign SPA shell (@webforms/player); no fillable Right-to-Know fields were confirmed (10 Sep 2026). Treat that URL as UNCONFIRMED. No Procurement/Public Works deputy ORO. Do not guess an email.</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
     <row r="1" ht="80" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Pilot: five Pennsylvania counties by FY2027 contracted tons. Primary recipient is the county Agency Open Records Officer (RTKL), verified 10 Sep 2026 from the county Right-to-Know page. Purchasing contacts are secondary only. Washington AORO email is UNVERIFIED (not published; use the county web form). Default: python scripts/pa_followup.py writes this workbook and .eml drafts. Sending requires --send and SALTTRACKER_FOLLOWUP_CONFIRM=YES and skips UNVERIFIED rows.</t>
+          <t>Pilot: five Pennsylvania counties by FY2027 contracted tons. Primary recipient is the county Agency Open Records Officer (RTKL), verified 10 Sep 2026 from the county Right-to-Know page. Purchasing contacts are secondary only. Washington AORO email is UNVERIFIED (not published; mail the Chief Clerk — the DocuSign link is unconfirmed). Default: python scripts/pa_followup.py writes this workbook and .eml drafts. Sending requires --send and SALTTRACKER_FOLLOWUP_CONFIRM=YES and skips UNVERIFIED rows.</t>
         </is>
       </c>
     </row>

</xml_diff>